<commit_message>
Belge yayın ve revizyon tarihlerini ana listeyle eşleştir
</commit_message>
<xml_diff>
--- a/EKG_Kalite_Yönetim_Sistemi/00_Yönetim Sistemi Çerçevesi/01_Kapsam, Süreçler ve Görevler/EKG-YNT-FRM-01_surec_kaplumbaga_diyagrami_her_surec_icin.xlsx
+++ b/EKG_Kalite_Yönetim_Sistemi/00_Yönetim Sistemi Çerçevesi/01_Kapsam, Süreçler ve Görevler/EKG-YNT-FRM-01_surec_kaplumbaga_diyagrami_her_surec_icin.xlsx
@@ -1398,7 +1398,8 @@
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="1">
     <x:oddHeader>&amp;L&amp;"Arial,Bold"&amp;11EKG-YNT-FRM-01&amp;C&amp;"Arial,Regular"&amp;11Süreç Kaplumbağa Diyagramı (her süreç için)</x:oddHeader>
-    <x:oddFooter>&amp;L&amp;"Arial,Regular"&amp;11İlk Yayın: 04.05.2026 | Revizyon: 19.10.2026&amp;R&amp;11Sayfa &amp;P / &amp;N</x:oddFooter>
+    <x:oddFooter>&amp;L&amp;"Arial,Regular"&amp;11İlk Yayın: 08.06.2026 | Revizyon: 14.09.2026
+Revizyon nedeni: Doküman kimliği ve ana liste ile tarih eşleşmesi güncellendi.&amp;R&amp;11Sayfa &amp;P / &amp;N</x:oddFooter>
   </x:headerFooter>
   <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02a5a1ed9bd4481b"/>
 </x:worksheet>
@@ -1601,7 +1602,8 @@
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="1">
     <x:oddHeader>&amp;L&amp;"Arial,Bold"&amp;11EKG-YNT-FRM-01&amp;C&amp;"Arial,Regular"&amp;11Süreç Kaplumbağa Diyagramı (her süreç için)</x:oddHeader>
-    <x:oddFooter>&amp;L&amp;"Arial,Regular"&amp;11İlk Yayın: 04.05.2026 | Revizyon: 19.10.2026&amp;R&amp;11Sayfa &amp;P / &amp;N</x:oddFooter>
+    <x:oddFooter>&amp;L&amp;"Arial,Regular"&amp;11İlk Yayın: 08.06.2026 | Revizyon: 14.09.2026
+Revizyon nedeni: Doküman kimliği ve ana liste ile tarih eşleşmesi güncellendi.&amp;R&amp;11Sayfa &amp;P / &amp;N</x:oddFooter>
   </x:headerFooter>
   <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3a5f54dd2e64f4b"/>
   <x:tableParts count="1">
@@ -1888,7 +1890,8 @@
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="1">
     <x:oddHeader>&amp;L&amp;"Arial,Bold"&amp;11EKG-YNT-FRM-01&amp;C&amp;"Arial,Regular"&amp;11Süreç Kaplumbağa Diyagramı (her süreç için)</x:oddHeader>
-    <x:oddFooter>&amp;L&amp;"Arial,Regular"&amp;11İlk Yayın: 04.05.2026 | Revizyon: 19.10.2026&amp;R&amp;11Sayfa &amp;P / &amp;N</x:oddFooter>
+    <x:oddFooter>&amp;L&amp;"Arial,Regular"&amp;11İlk Yayın: 08.06.2026 | Revizyon: 14.09.2026
+Revizyon nedeni: Doküman kimliği ve ana liste ile tarih eşleşmesi güncellendi.&amp;R&amp;11Sayfa &amp;P / &amp;N</x:oddFooter>
   </x:headerFooter>
   <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0164dd54263b408c"/>
   <x:tableParts count="1">
@@ -2132,7 +2135,8 @@
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="1">
     <x:oddHeader>&amp;L&amp;"Arial,Bold"&amp;11EKG-YNT-FRM-01&amp;C&amp;"Arial,Regular"&amp;11Süreç Kaplumbağa Diyagramı (her süreç için)</x:oddHeader>
-    <x:oddFooter>&amp;L&amp;"Arial,Regular"&amp;11İlk Yayın: 04.05.2026 | Revizyon: 19.10.2026&amp;R&amp;11Sayfa &amp;P / &amp;N</x:oddFooter>
+    <x:oddFooter>&amp;L&amp;"Arial,Regular"&amp;11İlk Yayın: 08.06.2026 | Revizyon: 14.09.2026
+Revizyon nedeni: Doküman kimliği ve ana liste ile tarih eşleşmesi güncellendi.&amp;R&amp;11Sayfa &amp;P / &amp;N</x:oddFooter>
   </x:headerFooter>
   <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R850ce7c5f2784ad7"/>
   <x:tableParts count="1">

</xml_diff>